<commit_message>
Final audit and fixes
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Waktu" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avalanche Effect" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shannon Entropy" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PBKDF2 KDF" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avalanche Effect" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shannon Entropy" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -539,22 +540,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>0.1578</v>
+        <v>0.1618</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.0071</v>
+        <v>0.0032</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.0026</v>
+        <v>0.0021</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.0027</v>
+        <v>0.0021</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.4673</v>
+        <v>0.4807</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.0156</v>
+        <v>0.0051</v>
       </c>
     </row>
     <row r="5">
@@ -569,22 +570,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.0167</v>
+        <v>0.0123</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.0045</v>
+        <v>0.0036</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.0031</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.0034</v>
+        <v>0.0029</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.0426</v>
+        <v>0.0304</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.0065</v>
+        <v>0.0049</v>
       </c>
     </row>
     <row r="6">
@@ -599,22 +600,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.6582</v>
+        <v>0.5163</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.6298</v>
+        <v>0.5295</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.5213</v>
+        <v>0.4798</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.5891999999999999</v>
+        <v>0.5155999999999999</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.7697000000000001</v>
+        <v>0.5365</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.6974</v>
+        <v>0.5553</v>
       </c>
     </row>
     <row r="7">
@@ -629,22 +630,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0.7963</v>
+        <v>0.8756</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.7112000000000001</v>
+        <v>0.7815</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.7534</v>
+        <v>0.7696</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0.6781</v>
+        <v>0.7638</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.8651</v>
+        <v>1.0626</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.7566000000000001</v>
+        <v>0.8126</v>
       </c>
     </row>
     <row r="8">
@@ -659,22 +660,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>4.9133</v>
+        <v>5.1428</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>4.5482</v>
+        <v>4.6228</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>4.3986</v>
+        <v>4.1638</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>4.1778</v>
+        <v>3.7989</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>5.6876</v>
+        <v>5.6796</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4.9601</v>
+        <v>5.7737</v>
       </c>
     </row>
     <row r="9">
@@ -689,22 +690,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>8.6</v>
+        <v>6.8191</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>8.0732</v>
+        <v>6.3647</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>8.402799999999999</v>
+        <v>5.9818</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>7.6491</v>
+        <v>6.0467</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>8.7468</v>
+        <v>7.2954</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>8.776400000000001</v>
+        <v>6.6982</v>
       </c>
     </row>
   </sheetData>
@@ -721,20 +722,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Algorithm</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Iterations</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Mean ms</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Min ms</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Max ms</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Stddev ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PBKDF2-HMAC-SHA256</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>600000</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>85.6284</v>
+      </c>
+      <c r="E2" t="n">
+        <v>84.0654</v>
+      </c>
+      <c r="F2" t="n">
+        <v>88.2907</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.892</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="64" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="51" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>HASIL PENGUJIAN AVALANCHE EFFECT (Perubahan 1 Bit Plaintext)</t>
+          <t>AVALANCHE EFFECT - CONTROLLED ONE-BIT MUTATIONS</t>
         </is>
       </c>
     </row>
@@ -747,22 +824,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Mutasi</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>Bit Berubah</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Total Bit</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Avalanche (%)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Target Ideal (%)</t>
         </is>
       </c>
     </row>
@@ -772,43 +849,89 @@
           <t>AES-256-GCM</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>63</v>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Plaintext bit</t>
+        </is>
       </c>
       <c r="C4" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>640</v>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>9.84%</t>
-        </is>
-      </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>11.56%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Key bit</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>337</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>640</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>52.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
           <t>ChaCha20-Poly1305</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>62</v>
-      </c>
-      <c r="C5" s="4" t="n">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Plaintext bit</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>640</v>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>9.69%</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>50.0%</t>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>9.84%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Key bit</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>317</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>640</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>49.53%</t>
         </is>
       </c>
     </row>
@@ -820,7 +943,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -873,12 +996,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>7.8113</t>
+          <t>7.8165</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>7.8273</t>
+          <t>7.8189</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -895,12 +1018,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>7.8113</t>
+          <t>7.8165</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>7.8097</t>
+          <t>7.7922</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">

</xml_diff>